<commit_message>
Add Austin Stone job info and the two Tex Air Austin orders
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014z5pCoVvnUESSHvBHrad3z
</commit_message>
<xml_diff>
--- a/tracker/Filter_Log.xlsx
+++ b/tracker/Filter_Log.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -449,7 +449,8 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -458,7 +459,11 @@
           <t>Job number</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>2250823</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -466,7 +471,11 @@
           <t>Project name</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Austin Stone</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -479,57 +488,88 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>PO number</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n"/>
+          <t>Airco PM</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Airco PM</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
           <t>Ordered by</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Angel Leon</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Filter size (W x L x D)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Qty per change</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Filter set installed</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>MERV</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Filter size (W x L x D)</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Qty per change</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>Filter set installed</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>RTU-1A</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>20x25x2</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>8</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Replaced</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -540,39 +580,49 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>20x25x2</t>
+          <t>20x20x2</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n"/>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>RTU-1A</t>
+          <t>RTU-2A</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>20x20x2</t>
+          <t>20x25x2</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n"/>
+      <c r="E10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -582,39 +632,49 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>20x25x2</t>
+          <t>20x20x2</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E11" s="2" t="n"/>
+      <c r="E11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>RTU-2A</t>
+          <t>RTU-1C</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>20x20x2</t>
+          <t>20x25x2</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E12" s="2" t="n"/>
+      <c r="E12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -624,39 +684,49 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>20x25x2</t>
+          <t>20x20x2</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E13" s="2" t="n"/>
+      <c r="E13" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>RTU-1C</t>
+          <t>RTU-2C</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>20x20x2</t>
+          <t>20x25x2</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E14" s="2" t="n"/>
+      <c r="E14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -666,39 +736,49 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>20x25x2</t>
+          <t>20x20x2</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E15" s="2" t="n"/>
+      <c r="E15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>RTU-2C</t>
+          <t>RTU-1B</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>20x20x2</t>
+          <t>20x25x4</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E16" s="2" t="n"/>
+      <c r="E16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -708,39 +788,49 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>20x25x4</t>
+          <t>20x20x4</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E17" s="2" t="n"/>
+      <c r="E17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>RTU-1B</t>
+          <t>RTU-2B-1</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>20x20x4</t>
+          <t>20x25x4</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E18" s="2" t="n"/>
+      <c r="E18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -750,39 +840,45 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>20x25x4</t>
+          <t>20x20x4</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="E19" s="2" t="n"/>
+      <c r="E19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>RTU-2B-1</t>
+          <t>RTU-2B-2</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>20x20x4</t>
+          <t>20x25x4</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>4</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Replaced</t>
+        <v>8</v>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Not replaced</t>
         </is>
       </c>
       <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -792,11 +888,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>20x25x4</t>
+          <t>20x20x4</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
@@ -804,16 +900,17 @@
         </is>
       </c>
       <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>RTU-2B-2</t>
+          <t>AHU-1</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>20x20x4</t>
+          <t>20x24x4</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -825,6 +922,7 @@
         </is>
       </c>
       <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -834,11 +932,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>20x24x4</t>
+          <t>20x20x4</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
@@ -846,16 +944,17 @@
         </is>
       </c>
       <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AHU-1</t>
+          <t>ERV-1</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>20x20x4</t>
+          <t>20x24x4</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -867,6 +966,7 @@
         </is>
       </c>
       <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -876,7 +976,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>20x24x4</t>
+          <t>16x20x4</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -888,6 +988,7 @@
         </is>
       </c>
       <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -897,7 +998,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>16x20x4</t>
+          <t>20x24x2</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -909,6 +1010,7 @@
         </is>
       </c>
       <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -918,7 +1020,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>20x24x2</t>
+          <t>16x24x2</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -930,27 +1032,7 @@
         </is>
       </c>
       <c r="E27" s="2" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>ERV-1</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>16x24x2</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>2</v>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>Not replaced</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>